<commit_message>
physique final et emploi du temps révision
</commit_message>
<xml_diff>
--- a/Emploi du temps.xlsx
+++ b/Emploi du temps.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gabin\Desktop\Dossiers\EPFL\BA2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FAB21FA-1C5D-4CBB-9791-32E6D6A5044C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27CCF3D2-B9FF-4107-B82D-3E8594D9BA21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{FC118514-611A-4C41-8D87-2DA3482F14D1}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="4" xr2:uid="{FC118514-611A-4C41-8D87-2DA3482F14D1}"/>
   </bookViews>
   <sheets>
     <sheet name="Emploi tu temps" sheetId="1" r:id="rId1"/>
     <sheet name="Séries" sheetId="4" r:id="rId2"/>
     <sheet name="Révisions a long terme" sheetId="2" r:id="rId3"/>
     <sheet name="Notes" sheetId="3" r:id="rId4"/>
+    <sheet name="Planning révision" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Emploi tu temps'!$B$2:$I$32</definedName>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="125">
   <si>
     <t>Heure</t>
   </si>
@@ -264,6 +265,159 @@
   </si>
   <si>
     <t>Séries refaites</t>
+  </si>
+  <si>
+    <t>Analyse</t>
+  </si>
+  <si>
+    <t>Physique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Algèbre </t>
+  </si>
+  <si>
+    <t>match</t>
+  </si>
+  <si>
+    <t>analyse</t>
+  </si>
+  <si>
+    <t>algèbre</t>
+  </si>
+  <si>
+    <t>physique</t>
+  </si>
+  <si>
+    <t>preuve et exercice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planning </t>
+  </si>
+  <si>
+    <t>Algèbre linéaire</t>
+  </si>
+  <si>
+    <t>chapitre</t>
+  </si>
+  <si>
+    <t>exo</t>
+  </si>
+  <si>
+    <t>thm</t>
+  </si>
+  <si>
+    <t>intégrale généralisée</t>
+  </si>
+  <si>
+    <t>Espace Rn</t>
+  </si>
+  <si>
+    <t>Fonctions</t>
+  </si>
+  <si>
+    <t>Dérivabilité</t>
+  </si>
+  <si>
+    <t>Dérivation supérieurs</t>
+  </si>
+  <si>
+    <t>intégrale paramètres</t>
+  </si>
+  <si>
+    <t>Difféomorphisme</t>
+  </si>
+  <si>
+    <t>Extrema</t>
+  </si>
+  <si>
+    <t>Intégrale Riemann</t>
+  </si>
+  <si>
+    <t>Equa diff</t>
+  </si>
+  <si>
+    <t>Polynôme</t>
+  </si>
+  <si>
+    <t>Valeurs propre</t>
+  </si>
+  <si>
+    <t>Forme billinéaire</t>
+  </si>
+  <si>
+    <t>Produit scalaire</t>
+  </si>
+  <si>
+    <t>Théorème spectral</t>
+  </si>
+  <si>
+    <t>équa diff</t>
+  </si>
+  <si>
+    <t>Jordan</t>
+  </si>
+  <si>
+    <t>Frobenius</t>
+  </si>
+  <si>
+    <t>Notion base</t>
+  </si>
+  <si>
+    <t>Fluide repos</t>
+  </si>
+  <si>
+    <t>Dynamique fluide</t>
+  </si>
+  <si>
+    <t>Ondes</t>
+  </si>
+  <si>
+    <t>Ondes dans fluide</t>
+  </si>
+  <si>
+    <t>Electrostatique</t>
+  </si>
+  <si>
+    <t>circuit électrique</t>
+  </si>
+  <si>
+    <t>magnétostatique</t>
+  </si>
+  <si>
+    <t>Induction</t>
+  </si>
+  <si>
+    <t>Maxwell</t>
+  </si>
+  <si>
+    <t>exo*</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>6 12 19</t>
+  </si>
+  <si>
+    <t>20 23 26</t>
+  </si>
+  <si>
+    <t>7 12 17</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>3 6 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 9 20 </t>
+  </si>
+  <si>
+    <t>8 18</t>
+  </si>
+  <si>
+    <t>7 9 10 24 28 46</t>
   </si>
 </sst>
 </file>
@@ -338,7 +492,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="19">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -443,12 +597,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="43">
+  <borders count="46">
     <border>
       <left/>
       <right/>
@@ -990,11 +1162,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="173">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1136,9 +1345,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1379,6 +1585,82 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1714,35 +1996,35 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CA73547-9859-48D3-9D0D-82A1A45BED28}">
   <dimension ref="B1:L32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="20.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="20.7265625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="16384" width="20.7109375" style="30"/>
+    <col min="1" max="16384" width="20.7265625" style="30"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="58" t="s">
+    <row r="1" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="57" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="59"/>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="I2" s="60"/>
-    </row>
-    <row r="3" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="61"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="62"/>
-      <c r="F3" s="62"/>
-      <c r="G3" s="62"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="63"/>
-    </row>
-    <row r="4" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="59"/>
+    </row>
+    <row r="3" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B3" s="60"/>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+      <c r="H3" s="61"/>
+      <c r="I3" s="62"/>
+    </row>
+    <row r="4" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B4" s="35" t="s">
         <v>0</v>
       </c>
@@ -1768,349 +2050,349 @@
         <v>67</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="89" t="s">
+    <row r="5" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="88" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="91"/>
-      <c r="D5" s="91"/>
-      <c r="E5" s="91"/>
-      <c r="F5" s="91"/>
-      <c r="G5" s="91"/>
-      <c r="H5" s="91"/>
-      <c r="I5" s="92"/>
-    </row>
-    <row r="6" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="90"/>
-      <c r="C6" s="93"/>
-      <c r="D6" s="93"/>
-      <c r="E6" s="93"/>
-      <c r="F6" s="93"/>
-      <c r="G6" s="93"/>
-      <c r="H6" s="93"/>
-      <c r="I6" s="94"/>
-    </row>
-    <row r="7" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="87" t="s">
+      <c r="C5" s="90"/>
+      <c r="D5" s="90"/>
+      <c r="E5" s="90"/>
+      <c r="F5" s="90"/>
+      <c r="G5" s="90"/>
+      <c r="H5" s="90"/>
+      <c r="I5" s="91"/>
+    </row>
+    <row r="6" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B6" s="89"/>
+      <c r="C6" s="92"/>
+      <c r="D6" s="92"/>
+      <c r="E6" s="92"/>
+      <c r="F6" s="92"/>
+      <c r="G6" s="92"/>
+      <c r="H6" s="92"/>
+      <c r="I6" s="93"/>
+    </row>
+    <row r="7" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="86" t="s">
         <v>14</v>
       </c>
       <c r="C7" s="33"/>
-      <c r="D7" s="99"/>
-      <c r="E7" s="124" t="s">
+      <c r="D7" s="98"/>
+      <c r="E7" s="123" t="s">
         <v>56</v>
       </c>
-      <c r="F7" s="97" t="s">
+      <c r="F7" s="96" t="s">
         <v>65</v>
       </c>
-      <c r="G7" s="97" t="s">
+      <c r="G7" s="96" t="s">
         <v>65</v>
       </c>
-      <c r="H7" s="101"/>
-      <c r="I7" s="65" t="s">
+      <c r="H7" s="100"/>
+      <c r="I7" s="64" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="88"/>
+    <row r="8" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B8" s="87"/>
       <c r="C8" s="33"/>
-      <c r="D8" s="100"/>
-      <c r="E8" s="124"/>
-      <c r="F8" s="98"/>
-      <c r="G8" s="98"/>
-      <c r="H8" s="102"/>
-      <c r="I8" s="65"/>
+      <c r="D8" s="99"/>
+      <c r="E8" s="123"/>
+      <c r="F8" s="97"/>
+      <c r="G8" s="97"/>
+      <c r="H8" s="101"/>
+      <c r="I8" s="64"/>
       <c r="K8" s="31"/>
       <c r="L8" s="32"/>
     </row>
-    <row r="9" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="87" t="s">
+    <row r="9" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="86" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="95" t="s">
+      <c r="C9" s="94" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="97" t="s">
+      <c r="D9" s="96" t="s">
         <v>65</v>
       </c>
-      <c r="E9" s="124"/>
-      <c r="F9" s="75"/>
-      <c r="G9" s="75"/>
-      <c r="H9" s="102"/>
-      <c r="I9" s="65"/>
-    </row>
-    <row r="10" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="88"/>
-      <c r="C10" s="96"/>
-      <c r="D10" s="98"/>
-      <c r="E10" s="125"/>
-      <c r="F10" s="76"/>
-      <c r="G10" s="76"/>
-      <c r="H10" s="102"/>
-      <c r="I10" s="65"/>
-    </row>
-    <row r="11" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="87" t="s">
+      <c r="E9" s="123"/>
+      <c r="F9" s="74"/>
+      <c r="G9" s="74"/>
+      <c r="H9" s="101"/>
+      <c r="I9" s="64"/>
+    </row>
+    <row r="10" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B10" s="87"/>
+      <c r="C10" s="95"/>
+      <c r="D10" s="97"/>
+      <c r="E10" s="124"/>
+      <c r="F10" s="75"/>
+      <c r="G10" s="75"/>
+      <c r="H10" s="101"/>
+      <c r="I10" s="64"/>
+    </row>
+    <row r="11" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="86" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="110" t="s">
+      <c r="C11" s="109" t="s">
         <v>54</v>
       </c>
-      <c r="D11" s="126" t="s">
+      <c r="D11" s="125" t="s">
         <v>55</v>
       </c>
-      <c r="E11" s="75"/>
-      <c r="F11" s="76"/>
-      <c r="G11" s="76"/>
-      <c r="H11" s="102"/>
-      <c r="I11" s="65"/>
+      <c r="E11" s="74"/>
+      <c r="F11" s="75"/>
+      <c r="G11" s="75"/>
+      <c r="H11" s="101"/>
+      <c r="I11" s="64"/>
       <c r="K11" s="30" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="88"/>
-      <c r="C12" s="111"/>
-      <c r="D12" s="127"/>
-      <c r="E12" s="76"/>
-      <c r="F12" s="76"/>
-      <c r="G12" s="76"/>
-      <c r="H12" s="102"/>
-      <c r="I12" s="65"/>
-    </row>
-    <row r="13" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="87" t="s">
+    <row r="12" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B12" s="87"/>
+      <c r="C12" s="110"/>
+      <c r="D12" s="126"/>
+      <c r="E12" s="75"/>
+      <c r="F12" s="75"/>
+      <c r="G12" s="75"/>
+      <c r="H12" s="101"/>
+      <c r="I12" s="64"/>
+    </row>
+    <row r="13" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="86" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="111"/>
-      <c r="D13" s="127"/>
-      <c r="E13" s="76"/>
-      <c r="F13" s="76"/>
-      <c r="G13" s="76"/>
-      <c r="H13" s="102"/>
-      <c r="I13" s="65"/>
-    </row>
-    <row r="14" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="88"/>
-      <c r="C14" s="112"/>
-      <c r="D14" s="128"/>
-      <c r="E14" s="77"/>
-      <c r="F14" s="77"/>
-      <c r="G14" s="77"/>
-      <c r="H14" s="102"/>
-      <c r="I14" s="66"/>
-    </row>
-    <row r="15" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="87" t="s">
+      <c r="C13" s="110"/>
+      <c r="D13" s="126"/>
+      <c r="E13" s="75"/>
+      <c r="F13" s="75"/>
+      <c r="G13" s="75"/>
+      <c r="H13" s="101"/>
+      <c r="I13" s="64"/>
+    </row>
+    <row r="14" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B14" s="87"/>
+      <c r="C14" s="111"/>
+      <c r="D14" s="127"/>
+      <c r="E14" s="76"/>
+      <c r="F14" s="76"/>
+      <c r="G14" s="76"/>
+      <c r="H14" s="101"/>
+      <c r="I14" s="65"/>
+    </row>
+    <row r="15" spans="2:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="86" t="s">
         <v>6</v>
       </c>
-      <c r="C15" s="81"/>
-      <c r="D15" s="82"/>
-      <c r="E15" s="82"/>
-      <c r="F15" s="82"/>
-      <c r="G15" s="83"/>
-      <c r="H15" s="102"/>
-      <c r="I15" s="104"/>
-    </row>
-    <row r="16" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="88"/>
-      <c r="C16" s="84"/>
-      <c r="D16" s="85"/>
-      <c r="E16" s="85"/>
-      <c r="F16" s="85"/>
-      <c r="G16" s="86"/>
-      <c r="H16" s="102"/>
-      <c r="I16" s="105"/>
-    </row>
-    <row r="17" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="87" t="s">
+      <c r="C15" s="80"/>
+      <c r="D15" s="81"/>
+      <c r="E15" s="81"/>
+      <c r="F15" s="81"/>
+      <c r="G15" s="82"/>
+      <c r="H15" s="101"/>
+      <c r="I15" s="103"/>
+    </row>
+    <row r="16" spans="2:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B16" s="87"/>
+      <c r="C16" s="83"/>
+      <c r="D16" s="84"/>
+      <c r="E16" s="84"/>
+      <c r="F16" s="84"/>
+      <c r="G16" s="85"/>
+      <c r="H16" s="101"/>
+      <c r="I16" s="104"/>
+    </row>
+    <row r="17" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="86" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="73"/>
-      <c r="D17" s="78" t="s">
+      <c r="C17" s="72"/>
+      <c r="D17" s="77" t="s">
         <v>59</v>
       </c>
-      <c r="E17" s="75"/>
-      <c r="F17" s="75"/>
-      <c r="G17" s="75"/>
-      <c r="H17" s="102"/>
-      <c r="I17" s="64" t="s">
+      <c r="E17" s="74"/>
+      <c r="F17" s="74"/>
+      <c r="G17" s="74"/>
+      <c r="H17" s="101"/>
+      <c r="I17" s="63" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="18" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="88"/>
-      <c r="C18" s="74"/>
-      <c r="D18" s="79"/>
-      <c r="E18" s="77"/>
-      <c r="F18" s="76"/>
-      <c r="G18" s="76"/>
-      <c r="H18" s="102"/>
-      <c r="I18" s="65"/>
-    </row>
-    <row r="19" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="87" t="s">
+    <row r="18" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B18" s="87"/>
+      <c r="C18" s="73"/>
+      <c r="D18" s="78"/>
+      <c r="E18" s="76"/>
+      <c r="F18" s="75"/>
+      <c r="G18" s="75"/>
+      <c r="H18" s="101"/>
+      <c r="I18" s="64"/>
+    </row>
+    <row r="19" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="86" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="74"/>
-      <c r="D19" s="121"/>
-      <c r="E19" s="78" t="s">
+      <c r="C19" s="73"/>
+      <c r="D19" s="120"/>
+      <c r="E19" s="77" t="s">
         <v>57</v>
       </c>
-      <c r="F19" s="76"/>
-      <c r="G19" s="76"/>
-      <c r="H19" s="102"/>
-      <c r="I19" s="65"/>
-    </row>
-    <row r="20" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="88"/>
-      <c r="C20" s="74"/>
-      <c r="D20" s="121"/>
-      <c r="E20" s="79"/>
-      <c r="F20" s="76"/>
-      <c r="G20" s="76"/>
-      <c r="H20" s="102"/>
-      <c r="I20" s="65"/>
-    </row>
-    <row r="21" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="87" t="s">
+      <c r="F19" s="75"/>
+      <c r="G19" s="75"/>
+      <c r="H19" s="101"/>
+      <c r="I19" s="64"/>
+    </row>
+    <row r="20" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B20" s="87"/>
+      <c r="C20" s="73"/>
+      <c r="D20" s="120"/>
+      <c r="E20" s="78"/>
+      <c r="F20" s="75"/>
+      <c r="G20" s="75"/>
+      <c r="H20" s="101"/>
+      <c r="I20" s="64"/>
+    </row>
+    <row r="21" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B21" s="86" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="74"/>
-      <c r="D21" s="122" t="s">
+      <c r="C21" s="73"/>
+      <c r="D21" s="121" t="s">
         <v>59</v>
       </c>
-      <c r="E21" s="79"/>
-      <c r="F21" s="76"/>
-      <c r="G21" s="76"/>
-      <c r="H21" s="102"/>
-      <c r="I21" s="65"/>
+      <c r="E21" s="78"/>
+      <c r="F21" s="75"/>
+      <c r="G21" s="75"/>
+      <c r="H21" s="101"/>
+      <c r="I21" s="64"/>
       <c r="K21" s="34"/>
     </row>
-    <row r="22" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="88"/>
-      <c r="C22" s="74"/>
-      <c r="D22" s="123"/>
-      <c r="E22" s="80"/>
-      <c r="F22" s="76"/>
-      <c r="G22" s="76"/>
-      <c r="H22" s="102"/>
-      <c r="I22" s="65"/>
-    </row>
-    <row r="23" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="87" t="s">
+    <row r="22" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B22" s="87"/>
+      <c r="C22" s="73"/>
+      <c r="D22" s="122"/>
+      <c r="E22" s="79"/>
+      <c r="F22" s="75"/>
+      <c r="G22" s="75"/>
+      <c r="H22" s="101"/>
+      <c r="I22" s="64"/>
+    </row>
+    <row r="23" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B23" s="86" t="s">
         <v>11</v>
       </c>
-      <c r="C23" s="74"/>
-      <c r="D23" s="71"/>
-      <c r="E23" s="119" t="s">
+      <c r="C23" s="73"/>
+      <c r="D23" s="70"/>
+      <c r="E23" s="118" t="s">
         <v>58</v>
       </c>
-      <c r="F23" s="76"/>
-      <c r="G23" s="76"/>
-      <c r="H23" s="102"/>
-      <c r="I23" s="65"/>
-    </row>
-    <row r="24" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="88"/>
-      <c r="C24" s="74"/>
-      <c r="D24" s="72"/>
-      <c r="E24" s="120"/>
-      <c r="F24" s="76"/>
-      <c r="G24" s="76"/>
-      <c r="H24" s="102"/>
-      <c r="I24" s="65"/>
-    </row>
-    <row r="25" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="87" t="s">
+      <c r="F23" s="75"/>
+      <c r="G23" s="75"/>
+      <c r="H23" s="101"/>
+      <c r="I23" s="64"/>
+    </row>
+    <row r="24" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B24" s="87"/>
+      <c r="C24" s="73"/>
+      <c r="D24" s="71"/>
+      <c r="E24" s="119"/>
+      <c r="F24" s="75"/>
+      <c r="G24" s="75"/>
+      <c r="H24" s="101"/>
+      <c r="I24" s="64"/>
+    </row>
+    <row r="25" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B25" s="86" t="s">
         <v>12</v>
       </c>
-      <c r="C25" s="74"/>
-      <c r="D25" s="72"/>
-      <c r="E25" s="71"/>
-      <c r="F25" s="76"/>
-      <c r="G25" s="76"/>
-      <c r="H25" s="102"/>
-      <c r="I25" s="65"/>
-    </row>
-    <row r="26" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="88"/>
-      <c r="C26" s="74"/>
-      <c r="D26" s="72"/>
-      <c r="E26" s="72"/>
-      <c r="F26" s="76"/>
-      <c r="G26" s="76"/>
-      <c r="H26" s="102"/>
-      <c r="I26" s="66"/>
-    </row>
-    <row r="27" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="89" t="s">
+      <c r="C25" s="73"/>
+      <c r="D25" s="71"/>
+      <c r="E25" s="70"/>
+      <c r="F25" s="75"/>
+      <c r="G25" s="75"/>
+      <c r="H25" s="101"/>
+      <c r="I25" s="64"/>
+    </row>
+    <row r="26" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B26" s="87"/>
+      <c r="C26" s="73"/>
+      <c r="D26" s="71"/>
+      <c r="E26" s="71"/>
+      <c r="F26" s="75"/>
+      <c r="G26" s="75"/>
+      <c r="H26" s="101"/>
+      <c r="I26" s="65"/>
+    </row>
+    <row r="27" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B27" s="88" t="s">
         <v>19</v>
       </c>
-      <c r="C27" s="106" t="s">
+      <c r="C27" s="105" t="s">
         <v>61</v>
       </c>
-      <c r="D27" s="106"/>
-      <c r="E27" s="106"/>
-      <c r="F27" s="106"/>
-      <c r="G27" s="107"/>
-      <c r="H27" s="102"/>
-      <c r="I27" s="117" t="s">
+      <c r="D27" s="105"/>
+      <c r="E27" s="105"/>
+      <c r="F27" s="105"/>
+      <c r="G27" s="106"/>
+      <c r="H27" s="101"/>
+      <c r="I27" s="116" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="28" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="90"/>
-      <c r="C28" s="108"/>
-      <c r="D28" s="108"/>
-      <c r="E28" s="108"/>
-      <c r="F28" s="108"/>
-      <c r="G28" s="109"/>
-      <c r="H28" s="102"/>
-      <c r="I28" s="118"/>
-    </row>
-    <row r="29" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="89" t="s">
+    <row r="28" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B28" s="89"/>
+      <c r="C28" s="107"/>
+      <c r="D28" s="107"/>
+      <c r="E28" s="107"/>
+      <c r="F28" s="107"/>
+      <c r="G28" s="108"/>
+      <c r="H28" s="101"/>
+      <c r="I28" s="117"/>
+    </row>
+    <row r="29" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B29" s="88" t="s">
         <v>17</v>
       </c>
-      <c r="C29" s="67"/>
-      <c r="D29" s="67"/>
-      <c r="E29" s="67"/>
-      <c r="F29" s="67"/>
-      <c r="G29" s="68"/>
-      <c r="H29" s="102"/>
+      <c r="C29" s="66"/>
+      <c r="D29" s="66"/>
+      <c r="E29" s="66"/>
+      <c r="F29" s="66"/>
+      <c r="G29" s="67"/>
+      <c r="H29" s="101"/>
       <c r="I29" s="28"/>
     </row>
-    <row r="30" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="90"/>
-      <c r="C30" s="69"/>
-      <c r="D30" s="69"/>
-      <c r="E30" s="69"/>
-      <c r="F30" s="69"/>
-      <c r="G30" s="70"/>
-      <c r="H30" s="103"/>
+    <row r="30" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B30" s="89"/>
+      <c r="C30" s="68"/>
+      <c r="D30" s="68"/>
+      <c r="E30" s="68"/>
+      <c r="F30" s="68"/>
+      <c r="G30" s="69"/>
+      <c r="H30" s="102"/>
       <c r="I30" s="29"/>
     </row>
-    <row r="31" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="64" t="s">
+    <row r="31" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B31" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="C31" s="113"/>
-      <c r="D31" s="113"/>
-      <c r="E31" s="113"/>
-      <c r="F31" s="113"/>
-      <c r="G31" s="113"/>
-      <c r="H31" s="113"/>
-      <c r="I31" s="114"/>
-    </row>
-    <row r="32" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="66"/>
-      <c r="C32" s="115"/>
-      <c r="D32" s="115"/>
-      <c r="E32" s="115"/>
-      <c r="F32" s="115"/>
-      <c r="G32" s="115"/>
-      <c r="H32" s="115"/>
-      <c r="I32" s="116"/>
+      <c r="C31" s="112"/>
+      <c r="D31" s="112"/>
+      <c r="E31" s="112"/>
+      <c r="F31" s="112"/>
+      <c r="G31" s="112"/>
+      <c r="H31" s="112"/>
+      <c r="I31" s="113"/>
+    </row>
+    <row r="32" spans="2:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B32" s="65"/>
+      <c r="C32" s="114"/>
+      <c r="D32" s="114"/>
+      <c r="E32" s="114"/>
+      <c r="F32" s="114"/>
+      <c r="G32" s="114"/>
+      <c r="H32" s="114"/>
+      <c r="I32" s="115"/>
     </row>
   </sheetData>
   <mergeCells count="46">
@@ -2170,52 +2452,52 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCBDDCAD-6C57-475E-A0BD-9133A1F72065}">
   <dimension ref="B1:R18"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="9" max="9" width="13.7109375" customWidth="1"/>
-    <col min="10" max="10" width="13.85546875" customWidth="1"/>
+    <col min="9" max="9" width="13.7265625" customWidth="1"/>
+    <col min="10" max="10" width="13.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B2" s="52" t="s">
+    <row r="1" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:18" x14ac:dyDescent="0.35">
+      <c r="B2" s="51" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="54"/>
-      <c r="H2" s="52" t="s">
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="53"/>
+      <c r="H2" s="51" t="s">
         <v>73</v>
       </c>
-      <c r="I2" s="53"/>
-      <c r="J2" s="53"/>
-      <c r="K2" s="53"/>
-      <c r="L2" s="54"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
+      <c r="K2" s="52"/>
+      <c r="L2" s="53"/>
       <c r="M2" s="5"/>
       <c r="N2" s="5"/>
       <c r="P2" s="5"/>
       <c r="Q2" s="5"/>
       <c r="R2" s="5"/>
     </row>
-    <row r="3" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="55"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="57"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="56"/>
-      <c r="K3" s="56"/>
-      <c r="L3" s="57"/>
+    <row r="3" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B3" s="54"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="56"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="55"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="55"/>
+      <c r="L3" s="56"/>
       <c r="M3" s="44"/>
       <c r="N3" s="45"/>
       <c r="P3" s="50"/>
       <c r="Q3" s="44"/>
       <c r="R3" s="45"/>
     </row>
-    <row r="4" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B4" s="12" t="s">
         <v>62</v>
       </c>
@@ -2247,7 +2529,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B5" s="16">
         <v>1</v>
       </c>
@@ -2263,7 +2545,7 @@
       <c r="K5" s="48"/>
       <c r="L5" s="49"/>
     </row>
-    <row r="6" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B6" s="17">
         <v>2</v>
       </c>
@@ -2279,7 +2561,7 @@
       <c r="K6" s="41"/>
       <c r="L6" s="42"/>
     </row>
-    <row r="7" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B7" s="17">
         <v>3</v>
       </c>
@@ -2295,7 +2577,7 @@
       <c r="K7" s="41"/>
       <c r="L7" s="42"/>
     </row>
-    <row r="8" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B8" s="17">
         <v>4</v>
       </c>
@@ -2311,7 +2593,7 @@
       <c r="K8" s="41"/>
       <c r="L8" s="42"/>
     </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B9" s="17">
         <v>5</v>
       </c>
@@ -2327,7 +2609,7 @@
       <c r="K9" s="41"/>
       <c r="L9" s="42"/>
     </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B10" s="17">
         <v>6</v>
       </c>
@@ -2347,7 +2629,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B11" s="17">
         <v>7</v>
       </c>
@@ -2363,7 +2645,7 @@
       <c r="K11" s="2"/>
       <c r="L11" s="46"/>
     </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B12" s="17">
         <v>8</v>
       </c>
@@ -2379,14 +2661,14 @@
       <c r="K12" s="2"/>
       <c r="L12" s="19"/>
     </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B13" s="17">
         <v>9</v>
       </c>
       <c r="C13" s="25"/>
       <c r="D13" s="26"/>
       <c r="E13" s="26"/>
-      <c r="F13" s="51"/>
+      <c r="F13" s="42"/>
       <c r="H13" s="17">
         <v>9</v>
       </c>
@@ -2395,7 +2677,7 @@
       <c r="K13" s="2"/>
       <c r="L13" s="19"/>
     </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B14" s="17">
         <v>10</v>
       </c>
@@ -2411,7 +2693,7 @@
       <c r="K14" s="2"/>
       <c r="L14" s="19"/>
     </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B15" s="17">
         <v>11</v>
       </c>
@@ -2427,12 +2709,12 @@
       <c r="K15" s="2"/>
       <c r="L15" s="19"/>
     </row>
-    <row r="16" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B16" s="17">
         <v>12</v>
       </c>
-      <c r="C16" s="43"/>
-      <c r="D16" s="41"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="26"/>
       <c r="E16" s="26"/>
       <c r="F16" s="42"/>
       <c r="H16" s="17">
@@ -2443,7 +2725,7 @@
       <c r="K16" s="2"/>
       <c r="L16" s="19"/>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
       <c r="B17" s="17">
         <v>13</v>
       </c>
@@ -2459,7 +2741,7 @@
       <c r="K17" s="2"/>
       <c r="L17" s="19"/>
     </row>
-    <row r="18" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B18" s="20">
         <v>14</v>
       </c>
@@ -2487,32 +2769,32 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A00B4DD-F7F4-4A2A-854F-AB42A4A36BF8}">
   <dimension ref="B2:Q17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="16384" width="11.453125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B2" s="129" t="s">
+    <row r="2" spans="2:17" x14ac:dyDescent="0.35">
+      <c r="B2" s="128" t="s">
         <v>53</v>
       </c>
-      <c r="C2" s="130"/>
-      <c r="D2" s="130"/>
-      <c r="E2" s="130"/>
-      <c r="F2" s="130"/>
-      <c r="G2" s="130"/>
-      <c r="H2" s="130"/>
-      <c r="I2" s="130"/>
-      <c r="J2" s="130"/>
-      <c r="K2" s="130"/>
-      <c r="L2" s="130"/>
-      <c r="M2" s="130"/>
-      <c r="N2" s="130"/>
-      <c r="O2" s="130"/>
-      <c r="P2" s="130"/>
-      <c r="Q2" s="131"/>
-    </row>
-    <row r="3" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="C2" s="129"/>
+      <c r="D2" s="129"/>
+      <c r="E2" s="129"/>
+      <c r="F2" s="129"/>
+      <c r="G2" s="129"/>
+      <c r="H2" s="129"/>
+      <c r="I2" s="129"/>
+      <c r="J2" s="129"/>
+      <c r="K2" s="129"/>
+      <c r="L2" s="129"/>
+      <c r="M2" s="129"/>
+      <c r="N2" s="129"/>
+      <c r="O2" s="129"/>
+      <c r="P2" s="129"/>
+      <c r="Q2" s="130"/>
+    </row>
+    <row r="3" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
         <v>21</v>
       </c>
@@ -2534,7 +2816,7 @@
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
     </row>
-    <row r="4" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>22</v>
       </c>
@@ -2558,7 +2840,7 @@
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
     </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B5" s="3" t="s">
         <v>23</v>
       </c>
@@ -2582,7 +2864,7 @@
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
     </row>
-    <row r="6" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>24</v>
       </c>
@@ -2608,7 +2890,7 @@
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
     </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>25</v>
       </c>
@@ -2634,7 +2916,7 @@
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
     </row>
-    <row r="8" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B8" s="3" t="s">
         <v>26</v>
       </c>
@@ -2660,7 +2942,7 @@
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
     </row>
-    <row r="9" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B9" s="3" t="s">
         <v>27</v>
       </c>
@@ -2686,7 +2968,7 @@
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
     </row>
-    <row r="10" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B10" s="3" t="s">
         <v>28</v>
       </c>
@@ -2714,7 +2996,7 @@
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
     </row>
-    <row r="11" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B11" s="3" t="s">
         <v>29</v>
       </c>
@@ -2742,7 +3024,7 @@
       <c r="P11" s="4"/>
       <c r="Q11" s="4"/>
     </row>
-    <row r="12" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B12" s="3" t="s">
         <v>30</v>
       </c>
@@ -2770,7 +3052,7 @@
       <c r="P12" s="4"/>
       <c r="Q12" s="4"/>
     </row>
-    <row r="13" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B13" s="3" t="s">
         <v>31</v>
       </c>
@@ -2798,7 +3080,7 @@
       <c r="P13" s="4"/>
       <c r="Q13" s="4"/>
     </row>
-    <row r="14" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B14" s="3" t="s">
         <v>32</v>
       </c>
@@ -2826,7 +3108,7 @@
       <c r="P14" s="4"/>
       <c r="Q14" s="4"/>
     </row>
-    <row r="15" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B15" s="3" t="s">
         <v>33</v>
       </c>
@@ -2856,7 +3138,7 @@
       <c r="P15" s="4"/>
       <c r="Q15" s="4"/>
     </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B16" s="3" t="s">
         <v>34</v>
       </c>
@@ -2888,7 +3170,7 @@
       </c>
       <c r="Q16" s="4"/>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
     </row>
@@ -2904,9 +3186,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70A99AB2-D791-4B39-AC5C-775A72418923}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="16" x14ac:dyDescent="0.4">
       <c r="A1" s="6" t="s">
         <v>35</v>
       </c>
@@ -2930,7 +3212,7 @@
       </c>
       <c r="H1" s="6"/>
     </row>
-    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="16" x14ac:dyDescent="0.4">
       <c r="A2" s="6" t="s">
         <v>42</v>
       </c>
@@ -2957,7 +3239,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="16" x14ac:dyDescent="0.4">
       <c r="A3" s="6" t="s">
         <v>43</v>
       </c>
@@ -2971,17 +3253,17 @@
         <v>4.25</v>
       </c>
       <c r="E3" s="6">
-        <v>3.25</v>
-      </c>
-      <c r="F3" s="6">
-        <v>1.75</v>
+        <v>5.5</v>
+      </c>
+      <c r="F3" s="131">
+        <v>5.5</v>
       </c>
       <c r="G3" s="6">
-        <v>2.75</v>
+        <v>5.5</v>
       </c>
       <c r="H3" s="6"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>44</v>
       </c>
@@ -2999,22 +3281,22 @@
       </c>
       <c r="E4" s="7">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="F4" s="7">
         <f t="shared" si="0"/>
-        <v>12.25</v>
+        <v>38.5</v>
       </c>
       <c r="G4" s="7">
-        <f t="shared" si="0"/>
-        <v>13.75</v>
+        <f>G2*G3</f>
+        <v>27.5</v>
       </c>
       <c r="H4" s="7">
         <f>SUM(B4:G4)</f>
-        <v>162.25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="19.5" x14ac:dyDescent="0.3">
+        <v>220.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -3026,10 +3308,10 @@
       </c>
       <c r="H6" s="9">
         <f>H4/H2</f>
-        <v>3.9573170731707319</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+        <v>5.3719512195121952</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="16" x14ac:dyDescent="0.4">
       <c r="A8" s="6" t="s">
         <v>35</v>
       </c>
@@ -3051,7 +3333,7 @@
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
     </row>
-    <row r="9" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="16" x14ac:dyDescent="0.4">
       <c r="A9" s="6" t="s">
         <v>42</v>
       </c>
@@ -3076,7 +3358,7 @@
       </c>
       <c r="H9" s="6"/>
     </row>
-    <row r="10" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="16" x14ac:dyDescent="0.4">
       <c r="A10" s="6" t="s">
         <v>43</v>
       </c>
@@ -3098,7 +3380,7 @@
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
         <v>44</v>
       </c>
@@ -3128,7 +3410,7 @@
       </c>
       <c r="H11" s="7"/>
     </row>
-    <row r="13" spans="1:8" ht="19.5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="19.5" x14ac:dyDescent="0.45">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -3143,16 +3425,418 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="19.5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="19.5" x14ac:dyDescent="0.45">
       <c r="G15" s="10" t="s">
         <v>52</v>
       </c>
       <c r="H15" s="9">
         <f>(H4+G11)/(H2+G9)</f>
-        <v>4.0368852459016393</v>
+        <v>4.9877049180327866</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C89F3228-57D0-42A2-8574-2F5662BD37B3}">
+  <dimension ref="B1:N24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="17.36328125" customWidth="1"/>
+    <col min="4" max="4" width="19.54296875" customWidth="1"/>
+    <col min="5" max="5" width="19.1796875" customWidth="1"/>
+    <col min="6" max="6" width="17.453125" customWidth="1"/>
+    <col min="7" max="7" width="18.81640625" customWidth="1"/>
+    <col min="8" max="8" width="18.7265625" customWidth="1"/>
+    <col min="9" max="9" width="11.81640625" customWidth="1"/>
+    <col min="10" max="10" width="17.36328125" customWidth="1"/>
+    <col min="11" max="11" width="17" customWidth="1"/>
+    <col min="13" max="13" width="10.81640625" customWidth="1"/>
+    <col min="14" max="14" width="16.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="142" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" s="143"/>
+      <c r="D2" s="143"/>
+      <c r="E2" s="143"/>
+      <c r="F2" s="143"/>
+      <c r="G2" s="143"/>
+      <c r="H2" s="143"/>
+      <c r="I2" s="144"/>
+      <c r="K2" s="132" t="s">
+        <v>78</v>
+      </c>
+      <c r="L2" s="134" t="s">
+        <v>79</v>
+      </c>
+      <c r="M2" s="133" t="s">
+        <v>80</v>
+      </c>
+      <c r="N2" s="135" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B3" s="145"/>
+      <c r="C3" s="141" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="141" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="141" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" s="141" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="141" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" s="141" t="s">
+        <v>66</v>
+      </c>
+      <c r="I3" s="146" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B4" s="18">
+        <v>1</v>
+      </c>
+      <c r="C4" s="136"/>
+      <c r="D4" s="136"/>
+      <c r="E4" s="137"/>
+      <c r="F4" s="137" t="s">
+        <v>77</v>
+      </c>
+      <c r="G4" s="138"/>
+      <c r="H4" s="137"/>
+      <c r="I4" s="147"/>
+    </row>
+    <row r="5" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B5" s="18">
+        <v>2</v>
+      </c>
+      <c r="C5" s="137"/>
+      <c r="D5" s="139"/>
+      <c r="E5" s="139"/>
+      <c r="F5" s="139"/>
+      <c r="G5" s="138"/>
+      <c r="H5" s="139"/>
+      <c r="I5" s="27" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B6" s="18">
+        <v>3</v>
+      </c>
+      <c r="C6" s="26"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="138"/>
+      <c r="H6" s="137"/>
+      <c r="I6" s="147"/>
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B7" s="18">
+        <v>4</v>
+      </c>
+      <c r="C7" s="137"/>
+      <c r="D7" s="140" t="s">
+        <v>74</v>
+      </c>
+      <c r="E7" s="139"/>
+      <c r="F7" s="139"/>
+      <c r="G7" s="140" t="s">
+        <v>75</v>
+      </c>
+      <c r="H7" s="26"/>
+      <c r="I7" s="27"/>
+    </row>
+    <row r="8" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B8" s="21">
+        <v>5</v>
+      </c>
+      <c r="C8" s="148" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
+      <c r="I8" s="23"/>
+    </row>
+    <row r="9" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B10" s="160" t="s">
+        <v>74</v>
+      </c>
+      <c r="C10" s="161"/>
+      <c r="D10" s="162"/>
+      <c r="E10" s="149"/>
+      <c r="F10" s="160" t="s">
+        <v>83</v>
+      </c>
+      <c r="G10" s="161"/>
+      <c r="H10" s="162"/>
+      <c r="J10" s="160" t="s">
+        <v>75</v>
+      </c>
+      <c r="K10" s="162"/>
+      <c r="L10" s="163"/>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B11" s="165" t="s">
+        <v>84</v>
+      </c>
+      <c r="C11" s="166" t="s">
+        <v>85</v>
+      </c>
+      <c r="D11" s="167" t="s">
+        <v>86</v>
+      </c>
+      <c r="E11" s="149"/>
+      <c r="F11" s="157" t="s">
+        <v>84</v>
+      </c>
+      <c r="G11" s="158" t="s">
+        <v>85</v>
+      </c>
+      <c r="H11" s="159" t="s">
+        <v>115</v>
+      </c>
+      <c r="J11" s="155" t="s">
+        <v>84</v>
+      </c>
+      <c r="K11" s="152" t="s">
+        <v>85</v>
+      </c>
+      <c r="L11" s="149"/>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B12" s="168" t="s">
+        <v>87</v>
+      </c>
+      <c r="C12" s="169"/>
+      <c r="D12" s="164" t="s">
+        <v>116</v>
+      </c>
+      <c r="E12" s="149"/>
+      <c r="F12" s="155" t="s">
+        <v>97</v>
+      </c>
+      <c r="G12" s="150"/>
+      <c r="H12" s="152"/>
+      <c r="J12" s="155" t="s">
+        <v>105</v>
+      </c>
+      <c r="K12" s="152"/>
+      <c r="L12" s="149"/>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B13" s="168" t="s">
+        <v>88</v>
+      </c>
+      <c r="C13" s="169"/>
+      <c r="D13" s="164" t="s">
+        <v>117</v>
+      </c>
+      <c r="E13" s="149"/>
+      <c r="F13" s="155" t="s">
+        <v>98</v>
+      </c>
+      <c r="G13" s="150"/>
+      <c r="H13" s="152"/>
+      <c r="J13" s="155" t="s">
+        <v>106</v>
+      </c>
+      <c r="K13" s="152"/>
+      <c r="L13" s="149"/>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B14" s="168" t="s">
+        <v>89</v>
+      </c>
+      <c r="C14" s="169"/>
+      <c r="D14" s="164" t="s">
+        <v>118</v>
+      </c>
+      <c r="E14" s="149"/>
+      <c r="F14" s="155" t="s">
+        <v>99</v>
+      </c>
+      <c r="G14" s="150"/>
+      <c r="H14" s="152"/>
+      <c r="J14" s="155" t="s">
+        <v>107</v>
+      </c>
+      <c r="K14" s="152"/>
+      <c r="L14" s="149"/>
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B15" s="168" t="s">
+        <v>90</v>
+      </c>
+      <c r="C15" s="169"/>
+      <c r="D15" s="164" t="s">
+        <v>119</v>
+      </c>
+      <c r="E15" s="149"/>
+      <c r="F15" s="155" t="s">
+        <v>100</v>
+      </c>
+      <c r="G15" s="150"/>
+      <c r="H15" s="152"/>
+      <c r="J15" s="155" t="s">
+        <v>108</v>
+      </c>
+      <c r="K15" s="152"/>
+      <c r="L15" s="149"/>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B16" s="168" t="s">
+        <v>91</v>
+      </c>
+      <c r="C16" s="169"/>
+      <c r="D16" s="164" t="s">
+        <v>120</v>
+      </c>
+      <c r="E16" s="149"/>
+      <c r="F16" s="155" t="s">
+        <v>101</v>
+      </c>
+      <c r="G16" s="150"/>
+      <c r="H16" s="152"/>
+      <c r="J16" s="155" t="s">
+        <v>109</v>
+      </c>
+      <c r="K16" s="152"/>
+      <c r="L16" s="149"/>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B17" s="168" t="s">
+        <v>92</v>
+      </c>
+      <c r="C17" s="169"/>
+      <c r="D17" s="164" t="s">
+        <v>121</v>
+      </c>
+      <c r="E17" s="149"/>
+      <c r="F17" s="155" t="s">
+        <v>102</v>
+      </c>
+      <c r="G17" s="150"/>
+      <c r="H17" s="152"/>
+      <c r="J17" s="155" t="s">
+        <v>110</v>
+      </c>
+      <c r="K17" s="152"/>
+      <c r="L17" s="149"/>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B18" s="168" t="s">
+        <v>93</v>
+      </c>
+      <c r="C18" s="169"/>
+      <c r="D18" s="164" t="s">
+        <v>122</v>
+      </c>
+      <c r="E18" s="149"/>
+      <c r="F18" s="155" t="s">
+        <v>103</v>
+      </c>
+      <c r="G18" s="150"/>
+      <c r="H18" s="152"/>
+      <c r="J18" s="155" t="s">
+        <v>111</v>
+      </c>
+      <c r="K18" s="152"/>
+      <c r="L18" s="149"/>
+    </row>
+    <row r="19" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B19" s="168" t="s">
+        <v>94</v>
+      </c>
+      <c r="C19" s="169"/>
+      <c r="D19" s="164" t="s">
+        <v>123</v>
+      </c>
+      <c r="E19" s="149"/>
+      <c r="F19" s="156" t="s">
+        <v>104</v>
+      </c>
+      <c r="G19" s="153"/>
+      <c r="H19" s="154"/>
+      <c r="J19" s="155" t="s">
+        <v>112</v>
+      </c>
+      <c r="K19" s="152"/>
+      <c r="L19" s="149"/>
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B20" s="168" t="s">
+        <v>95</v>
+      </c>
+      <c r="C20" s="169"/>
+      <c r="D20" s="164" t="s">
+        <v>124</v>
+      </c>
+      <c r="E20" s="149"/>
+      <c r="J20" s="155" t="s">
+        <v>113</v>
+      </c>
+      <c r="K20" s="152"/>
+      <c r="L20" s="149"/>
+    </row>
+    <row r="21" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B21" s="170" t="s">
+        <v>96</v>
+      </c>
+      <c r="C21" s="171"/>
+      <c r="D21" s="172"/>
+      <c r="E21" s="149"/>
+      <c r="J21" s="156" t="s">
+        <v>114</v>
+      </c>
+      <c r="K21" s="154"/>
+      <c r="L21" s="149"/>
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B22" s="151"/>
+      <c r="C22" s="149"/>
+      <c r="D22" s="149"/>
+      <c r="E22" s="149"/>
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B23" s="151"/>
+      <c r="C23" s="149"/>
+      <c r="D23" s="149"/>
+      <c r="E23" s="149"/>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B24" s="151"/>
+      <c r="C24" s="149"/>
+      <c r="D24" s="149"/>
+      <c r="E24" s="149"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="F10:H10"/>
+    <mergeCell ref="J10:K10"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>